<commit_message>
Add scripts for processing STIX files and extracting soil parameters
</commit_message>
<xml_diff>
--- a/attempts_tracking.xlsx
+++ b/attempts_tracking.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,26 @@
           <t>FoS_pernio_double_stage_tanphi_aso_bigger_DSS_updatedpar</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>FoS_bergambacht_reviewed</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>FoS_eemdijk_layeradjustment</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>FoS_ijkdijk_7a_AvD_refined</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>FoS_pernio_</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -507,6 +527,10 @@
         <v>0.4914564918851418</v>
       </c>
       <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -547,6 +571,10 @@
         <v>0.4914564918851418</v>
       </c>
       <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -587,6 +615,10 @@
         <v>0.4914564918851418</v>
       </c>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -629,6 +661,10 @@
       <c r="J5" t="n">
         <v>0.9537201397626098</v>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -669,6 +705,10 @@
         <v>0.4914564918851418</v>
       </c>
       <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -711,6 +751,10 @@
       <c r="J7" t="n">
         <v>0.9537201397626098</v>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -753,6 +797,10 @@
       <c r="J8" t="n">
         <v>0.9537201397626098</v>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -795,6 +843,10 @@
       <c r="J9" t="n">
         <v>0.9537201397626098</v>
       </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -831,6 +883,10 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -873,6 +929,10 @@
       <c r="J11" t="n">
         <v>0.9537201397626098</v>
       </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -915,6 +975,10 @@
       <c r="J12" t="n">
         <v>0.9149537727100676</v>
       </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -956,6 +1020,60 @@
       </c>
       <c r="J13" t="n">
         <v>0.9537201397626098</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Original baseline models - no modifications</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-04-14 11:59:43</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>UPLIFTVAN</t>
+        </is>
+      </c>
+      <c r="F14" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Run baseline models as-is to establish reference FoS</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>0.931843481075606</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>0.8533937238898434</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1.00092093909914</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.958105488603373</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0.9149537727100676</v>
       </c>
     </row>
   </sheetData>

</xml_diff>